<commit_message>
Adjust GUI size and simplify file label
Reduce main window height from 650 to 450 for a more compact layout and simplify the selected-file label to display only the filename (removed the leading "Selected "). Also includes an updated sample Excel workbook and an added Excel temporary/lock file (~$Synthesized_100_Six_Digit_Numbers.xlsx) — consider removing the temp file from the repo if it was added accidentally.
</commit_message>
<xml_diff>
--- a/sample_data/Synthesized_100_Six_Digit_Numbers.xlsx
+++ b/sample_data/Synthesized_100_Six_Digit_Numbers.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Programs\VSCODE Programs\GitHub\ERP_Automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Programs\VSCODE Programs\GitHub\ERP_RollUp_Automation\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3796BED9-230C-4253-8866-CE21C424688D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F2E78E-A73F-424F-B482-159FA2BA1C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="480" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,10 +22,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -363,165 +359,165 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A100"/>
+  <dimension ref="A1:B100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1">
         <v>473129</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>602734</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>711686</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>602808</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>745333</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>786237</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>994348</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>495179</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>998187</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>986441</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>951745</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>715028</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>451905</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>672716</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>714575</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <v>479291</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B16">
         <v>196331</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B17">
         <v>555341</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B18">
         <v>501252</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B19">
         <v>374976</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B20">
         <v>118469</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B21">
         <v>649441</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B22">
         <v>561661</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B23">
         <v>582416</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B24">
         <v>688459</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>117635</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>142902</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>354534</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>838491</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>535929</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>888097</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>814075</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>872082</v>
       </c>

</xml_diff>

<commit_message>
Add stop control and interrupt support to automation
Wire up a stop mechanism for the automation flow: run_automation now accepts stop_event and on_stopped, checks the event during countdown and processing, and reports processed count when interrupted. GUI updates: added a Stop button, threading.Event stop_event, stop_clicked handler, on_stopped callback, and start/stop state/styling changes; improved some labels and cursor hints. This enables graceful interruption of ongoing runs and updates UI accordingly.
</commit_message>
<xml_diff>
--- a/sample_data/Synthesized_100_Six_Digit_Numbers.xlsx
+++ b/sample_data/Synthesized_100_Six_Digit_Numbers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Programs\VSCODE Programs\GitHub\ERP_RollUp_Automation\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F2E78E-A73F-424F-B482-159FA2BA1C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB95927C-2B5C-4FC1-A96B-EC43EA7D1B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="480" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -442,423 +442,423 @@
         <v>196331</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>555341</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>501252</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>374976</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>118469</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>649441</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>561661</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23">
         <v>582416</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24">
         <v>688459</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B25">
         <v>117635</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B26">
         <v>142902</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B27">
         <v>354534</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B28">
         <v>838491</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B29">
         <v>535929</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B30">
         <v>888097</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B31">
         <v>814075</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B32">
         <v>872082</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B33">
         <v>403592</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B34">
         <v>248616</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B35">
         <v>121876</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B36">
         <v>872672</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B37">
         <v>341639</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B38">
         <v>101919</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B39">
         <v>339529</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B40">
         <v>225324</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B41">
         <v>419835</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B42">
         <v>833713</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B43">
         <v>882972</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B44">
         <v>935632</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B45">
         <v>450604</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B46">
         <v>884131</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B47">
         <v>452654</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B48">
         <v>578048</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B49">
         <v>475372</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B50">
         <v>966082</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B51">
         <v>467872</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B52">
         <v>897308</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B53">
         <v>374903</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B54">
         <v>903129</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B55">
         <v>819925</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B56">
         <v>922350</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B57">
         <v>114004</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B58">
         <v>255421</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B59">
         <v>847251</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B60">
         <v>480196</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B61">
         <v>166548</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B62">
         <v>234063</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B63">
         <v>666712</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B64">
         <v>904939</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B65">
         <v>716565</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66">
         <v>498546</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B67">
         <v>331026</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B68">
         <v>324859</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B69">
         <v>365919</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B70">
         <v>274266</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B71">
         <v>479291</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B72">
         <v>500208</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B73">
         <v>376164</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B74">
         <v>722048</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B75">
         <v>167233</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B76">
         <v>695468</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B77">
         <v>355708</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B78">
         <v>520998</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B79">
         <v>231106</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B80">
         <v>489344</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B81">
         <v>673901</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B82">
         <v>925244</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B83">
         <v>112084</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B84">
         <v>293423</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B85">
         <v>124359</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B86">
         <v>895679</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B87">
         <v>186470</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B88">
         <v>549535</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B89">
         <v>151718</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B90">
         <v>453933</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B91">
         <v>638181</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B92">
         <v>108922</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B93">
         <v>801595</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B94">
         <v>250071</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B95">
         <v>610077</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B96">
         <v>296951</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B97">
         <v>385151</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B98">
         <v>618007</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B99">
         <v>541429</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B100">
         <v>639818</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add watermark, update sample data and .gitignore
Add a small developer watermark label to the GUI (By Pranit Govande). Update sample_data: replace the 100-entry workbook, add Synthesized_500_Six_Digit_Numbers.xlsx, and remove the temporary ~$ file. Update .gitignore to include docs/ and clean up spacing. These changes add attribution and include a larger sample dataset.
</commit_message>
<xml_diff>
--- a/sample_data/Synthesized_100_Six_Digit_Numbers.xlsx
+++ b/sample_data/Synthesized_100_Six_Digit_Numbers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Programs\VSCODE Programs\GitHub\ERP_RollUp_Automation\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB95927C-2B5C-4FC1-A96B-EC43EA7D1B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F478A3F4-29EA-4D06-A1CA-61F4812058CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="480" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -408,7 +408,7 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="B10">
         <v>986441</v>
       </c>
     </row>
@@ -433,251 +433,251 @@
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B15">
-        <v>479291</v>
+      <c r="A15">
+        <v>714575</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B16">
+      <c r="A16">
         <v>196331</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>555341</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>501252</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>374976</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>118469</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B21">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>649441</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>561661</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B23">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>582416</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B24">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>688459</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>117635</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B26">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26">
         <v>142902</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B27">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>354534</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B28">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>838491</v>
       </c>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B29">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>535929</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B30">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>888097</v>
       </c>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B31">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31">
         <v>814075</v>
       </c>
     </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B32">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32">
         <v>872082</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B33">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33">
         <v>403592</v>
       </c>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B34">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34">
         <v>248616</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35">
         <v>121876</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B36">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36">
         <v>872672</v>
       </c>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B37">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37">
         <v>341639</v>
       </c>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B38">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38">
         <v>101919</v>
       </c>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B39">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39">
         <v>339529</v>
       </c>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B40">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40">
         <v>225324</v>
       </c>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B41">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41">
         <v>419835</v>
       </c>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B42">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42">
         <v>833713</v>
       </c>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B43">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43">
         <v>882972</v>
       </c>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B44">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44">
         <v>935632</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B45">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45">
         <v>450604</v>
       </c>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B46">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46">
         <v>884131</v>
       </c>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B47">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47">
         <v>452654</v>
       </c>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B48">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48">
         <v>578048</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B49">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49">
         <v>475372</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B50">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50">
         <v>966082</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B51">
         <v>467872</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B52">
         <v>897308</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B53">
         <v>374903</v>
       </c>
     </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B54">
         <v>903129</v>
       </c>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B55">
         <v>819925</v>
       </c>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B56">
         <v>922350</v>
       </c>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B57">
         <v>114004</v>
       </c>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B58">
         <v>255421</v>
       </c>
     </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B59">
         <v>847251</v>
       </c>
     </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B60">
         <v>480196</v>
       </c>
     </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B61">
         <v>166548</v>
       </c>
     </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B62">
         <v>234063</v>
       </c>
     </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B63">
         <v>666712</v>
       </c>
     </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B64">
         <v>904939</v>
       </c>

</xml_diff>